<commit_message>
Fix settings pill selector and update tracker sync to 98/100 completed
</commit_message>
<xml_diff>
--- a/youtube-automation/data/vehicles_tracker.xlsx
+++ b/youtube-automation/data/vehicles_tracker.xlsx
@@ -45,7 +45,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="007F6000"/>
+      <color rgb="00783F04"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -70,8 +70,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE5CD"/>
+        <bgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">

</xml_diff>